<commit_message>
Updates to testing files
</commit_message>
<xml_diff>
--- a/test/test_data/dj-specs-test.xlsx
+++ b/test/test_data/dj-specs-test.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\OnSSET\test\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Dokument\GitHub\MOZ-onsset\test\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{787DE35C-5023-4421-88D7-60C9C8B89BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="470" windowWidth="31460" windowHeight="10520" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioInfo" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="51">
   <si>
     <t>Scenario</t>
   </si>
@@ -156,13 +157,31 @@
   </si>
   <si>
     <t>dj</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>MaxIntensificationCost</t>
+  </si>
+  <si>
+    <t>CarbonTax</t>
+  </si>
+  <si>
+    <t>GridEmissionFactor</t>
+  </si>
+  <si>
+    <t>GridRenShare</t>
+  </si>
+  <si>
+    <t>ElecTarget</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,6 +201,11 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -226,7 +250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -238,10 +262,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -518,22 +545,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -562,7 +589,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -597,21 +624,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>9</v>
       </c>
@@ -645,8 +672,26 @@
       <c r="L1" t="s">
         <v>19</v>
       </c>
+      <c r="M1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>49</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -683,8 +728,26 @@
       <c r="L2">
         <v>0</v>
       </c>
+      <c r="M2">
+        <v>2500</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>4.2123221000000002E-2</v>
+      </c>
+      <c r="P2">
+        <v>766.03000789999999</v>
+      </c>
+      <c r="Q2">
+        <v>881.79840000000002</v>
+      </c>
+      <c r="R2">
+        <v>0.36752177800000002</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -721,8 +784,26 @@
       <c r="L3">
         <v>1</v>
       </c>
+      <c r="M3">
+        <v>2500</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>4.2123221000000002E-2</v>
+      </c>
+      <c r="P3">
+        <v>766.03000789999999</v>
+      </c>
+      <c r="Q3">
+        <v>881.79840000000002</v>
+      </c>
+      <c r="R3">
+        <v>0.36752177800000002</v>
+      </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -740,6 +821,24 @@
       </c>
       <c r="L4">
         <v>2</v>
+      </c>
+      <c r="M4">
+        <v>2500</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>4.2123221000000002E-2</v>
+      </c>
+      <c r="P4">
+        <v>766.03000789999999</v>
+      </c>
+      <c r="Q4">
+        <v>881.79840000000002</v>
+      </c>
+      <c r="R4">
+        <v>0.36752177800000002</v>
       </c>
     </row>
   </sheetData>
@@ -749,173 +848,262 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X2"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:AA3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1796875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="8.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.81640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.81640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="40.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.1796875" style="2" customWidth="1"/>
-    <col min="24" max="24" width="12.7265625" style="2" customWidth="1"/>
-    <col min="25" max="25" width="14.7265625" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.7265625" style="2" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="20" style="2" bestFit="1" customWidth="1"/>
-    <col min="31" max="50" width="9.1796875" style="2" customWidth="1"/>
-    <col min="51" max="16384" width="9.1796875" style="2"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="40.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="40.28515625" style="2" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.140625" style="2" customWidth="1"/>
+    <col min="27" max="27" width="12.7109375" style="2" customWidth="1"/>
+    <col min="28" max="28" width="14.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="20" style="2" bestFit="1" customWidth="1"/>
+    <col min="34" max="53" width="9.140625" style="2" customWidth="1"/>
+    <col min="54" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>2018</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>2030</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="G2" s="2">
         <v>971000</v>
       </c>
-      <c r="F2" s="2">
+      <c r="H2" s="2">
         <v>0.77800000000000002</v>
       </c>
-      <c r="I2" s="2">
+      <c r="K2" s="2">
         <v>1179150</v>
       </c>
-      <c r="J2" s="2">
+      <c r="L2" s="2">
         <v>0.8</v>
       </c>
-      <c r="K2" s="2">
+      <c r="M2" s="2">
         <v>7.7</v>
       </c>
-      <c r="L2" s="2">
+      <c r="N2" s="2">
         <v>6.5</v>
       </c>
-      <c r="M2" s="2">
+      <c r="O2" s="2">
         <v>4426</v>
       </c>
-      <c r="N2" s="2">
+      <c r="P2" s="2">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="O2" s="2">
+      <c r="Q2" s="2">
         <v>0.8</v>
       </c>
-      <c r="P2" s="2">
+      <c r="R2" s="2">
         <v>0.1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="S2" s="2">
         <v>50</v>
       </c>
-      <c r="R2" s="2">
+      <c r="T2" s="2">
         <v>19</v>
       </c>
-      <c r="S2" s="2">
+      <c r="U2" s="2">
+        <v>9999999</v>
+      </c>
+      <c r="V2" s="2">
         <v>0.6</v>
       </c>
-      <c r="T2" s="2">
+      <c r="W2" s="2">
         <v>0.26</v>
       </c>
-      <c r="U2" s="2">
+      <c r="X2" s="2">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2030</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2018</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2030</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2">
+        <v>971000</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0.77800000000000002</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1179150</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="M3" s="2">
+        <v>7.7</v>
+      </c>
+      <c r="N3" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="O3" s="2">
+        <v>4426</v>
+      </c>
+      <c r="P3" s="2">
+        <v>8.3000000000000004E-2</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="R3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="S3" s="2">
+        <v>50</v>
+      </c>
+      <c r="T3" s="2">
+        <v>19</v>
+      </c>
+      <c r="U3" s="2">
+        <v>9999999</v>
+      </c>
+      <c r="V3" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="W3" s="2">
+        <v>0.26</v>
+      </c>
+      <c r="X3" s="2">
         <v>0.7</v>
       </c>
     </row>

</xml_diff>